<commit_message>
etapa codificacion funcional hasta antes del analisis, falta herramientas
</commit_message>
<xml_diff>
--- a/output/xlsx/matriz_entrada_diseno.xlsx
+++ b/output/xlsx/matriz_entrada_diseno.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz de entrada" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matriz de entrada'!$A$1:$F$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matriz de entrada'!$A$1:$F$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -418,14 +418,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="47" customWidth="1" min="5" max="5"/>
     <col width="38" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -474,22 +474,22 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Consulta de horarios disponibles</t>
+          <t>Mostrar ejemplares disponibles para reserva</t>
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá consultar y mostrar únicamente los horarios disponibles de los médicos.</t>
+          <t>El sistema deberá mostrar únicamente los ejemplares que se encuentren disponibles para reserva.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>HU-001 – HU-001 - Consultar horarios disponibles</t>
+          <t>HU-001 – HU-001 - Reservar libro disponible</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Pendiente de definición y validación</t>
+          <t>Pendiente de validación</t>
         </is>
       </c>
     </row>
@@ -506,17 +506,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Visualización de datos del médico</t>
+          <t>Mostrar información del ejemplar antes de confirmar</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá mostrar el nombre y la especialidad del médico junto con los horarios disponibles.</t>
+          <t>El sistema deberá mostrar el título, autor, categoría y código del ejemplar antes de confirmar la reserva.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>HU-001 – HU-001 - Consultar horarios disponibles</t>
+          <t>HU-001 – HU-001 - Reservar libro disponible</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -538,49 +538,49 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Actualización de disponibilidad</t>
+          <t>Registrar reserva asociada al estudiante</t>
         </is>
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá actualizar la disponibilidad de horarios inmediatamente después de registrar una cita.</t>
+          <t>El sistema deberá registrar la reserva asociándola al estudiante autenticado, incluyendo el estudiante que realizó la reserva, el ejemplar seleccionado y la fecha y hora de la operación.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>HU-001 – HU-001 - Consultar horarios disponibles</t>
+          <t>HU-001 – HU-001 - Reservar libro disponible</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Pendiente de definición y validación</t>
+          <t>Pendiente de validación</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>RNF-001</t>
+          <t>RF-004</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>No funcional</t>
+          <t>Funcional</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Tiempo de respuesta de consulta</t>
+          <t>Cambiar estado del ejemplar a reservado</t>
         </is>
       </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá responder a la consulta de horarios disponibles en menos de tres segundos.</t>
+          <t>El sistema deberá cambiar el estado del ejemplar de disponible a reservado inmediatamente después de confirmar la reserva.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>HU-001 – HU-001 - Consultar horarios disponibles</t>
+          <t>HU-001 – HU-001 - Reservar libro disponible</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -592,27 +592,27 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>RNF-002</t>
+          <t>RF-005</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>No funcional</t>
+          <t>Funcional</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Visualización en tiempo real</t>
+          <t>Impedir reservas sobre ejemplares ya reservados</t>
         </is>
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá mostrar la información de horarios en tiempo real.</t>
+          <t>El sistema deberá impedir que otro estudiante reserve un ejemplar que ya tenga una reserva activa.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>HU-001 – HU-001 - Consultar horarios disponibles</t>
+          <t>HU-001 – HU-001 - Reservar libro disponible</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -624,7 +624,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>RF-004</t>
+          <t>RF-006</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -634,17 +634,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Registrar pacientes nuevos</t>
+          <t>Mostrar confirmación de reserva</t>
         </is>
       </c>
       <c r="D7" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá registrar pacientes nuevos.</t>
+          <t>El sistema deberá mostrar una confirmación cuando la reserva se registre correctamente.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>HU-002 – HU-002 - Registrar pacientes</t>
+          <t>HU-001 – HU-001 - Reservar libro disponible</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -656,7 +656,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>RF-005</t>
+          <t>RF-007</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -666,29 +666,29 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Validar documento de identidad</t>
+          <t>Informar fecha límite de recogida</t>
         </is>
       </c>
       <c r="D8" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá validar el documento de identidad del paciente.</t>
+          <t>El sistema deberá informar al estudiante la fecha límite establecida para recoger el ejemplar reservado.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>HU-002 – HU-002 - Registrar pacientes</t>
+          <t>HU-001 – HU-001 - Reservar libro disponible</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Pendiente de validación</t>
+          <t>Pendiente de definición y validación</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>RF-006</t>
+          <t>RF-008</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -698,29 +698,29 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Registrar información obligatoria</t>
+          <t>Actualización inmediata de disponibilidad</t>
         </is>
       </c>
       <c r="D9" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá registrar la información obligatoria del paciente.</t>
+          <t>El sistema deberá actualizar la disponibilidad inmediatamente después de confirmar una reserva.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>HU-002 – HU-002 - Registrar pacientes</t>
+          <t>HU-001 – HU-001 - Reservar libro disponible</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Pendiente de definición y validación</t>
+          <t>Pendiente de validación</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>RF-007</t>
+          <t>RF-009</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -730,17 +730,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Evitar registros duplicados</t>
+          <t>Un ejemplar solo puede tener una reserva activa simultáneamente</t>
         </is>
       </c>
       <c r="D10" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá evitar registros duplicados de pacientes.</t>
+          <t>El sistema deberá un ejemplar solo puede tener una reserva activa simultáneamente.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>HU-002 – HU-002 - Registrar pacientes</t>
+          <t>HU-001 – HU-001 - Reservar libro disponible</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -752,7 +752,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>RF-008</t>
+          <t>RF-010</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -762,29 +762,29 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Editar información del paciente</t>
+          <t>La reserva debe quedar asociada al estudiante que realizó la operación</t>
         </is>
       </c>
       <c r="D11" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá permitir editar posteriormente la información del paciente.</t>
+          <t>El sistema deberá la reserva debe quedar asociada al estudiante que realizó la operación.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>HU-002 – HU-002 - Registrar pacientes</t>
+          <t>HU-001 – HU-001 - Reservar libro disponible</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Pendiente de definición y validación</t>
+          <t>Pendiente de validación</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>RF-009</t>
+          <t>RF-011</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -794,17 +794,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Consultar agenda médica</t>
+          <t>La operación de reserva debe utilizar la disponibilidad actual del ejemplar. Se debe registrar el estudiante que realizó la reserva, el ejemplar seleccionado y la fecha y hora de la operación</t>
         </is>
       </c>
       <c r="D12" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá consultar la agenda médica mostrando las citas del día y el nombre del paciente.</t>
+          <t>El sistema deberá la operación de reserva debe utilizar la disponibilidad actual del ejemplar. Se debe registrar el estudiante que realizó la reserva, el ejemplar seleccionado y la fecha y hora de la operación.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>HU-003 – HU-003 - Consultar agenda médica</t>
+          <t>HU-001 – HU-001 - Reservar libro disponible</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -813,8 +813,296 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>RF-012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Registrar devolución de libro</t>
+        </is>
+      </c>
+      <c r="D13" s="1" t="inlineStr">
+        <is>
+          <t>El sistema deberá permitir registrar la devolución de un libro prestado.</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>HU-002 – HU-002 - Registrar préstamo de libro</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Pendiente de validación</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>RF-013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Verificar préstamo relacionado</t>
+        </is>
+      </c>
+      <c r="D14" s="1" t="inlineStr">
+        <is>
+          <t>El sistema deberá verificar que exista un préstamo relacionado con el libro al registrar su devolución.</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>HU-002 – HU-002 - Registrar préstamo de libro</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Pendiente de definición y validación</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>RF-014</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Actualizar información de préstamo</t>
+        </is>
+      </c>
+      <c r="D15" s="1" t="inlineStr">
+        <is>
+          <t>El sistema deberá actualizar la información del préstamo después de la devolución.</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>HU-002 – HU-002 - Registrar préstamo de libro</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Pendiente de definición y validación</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>RF-015</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Mostrar mensaje de confirmación de devolución</t>
+        </is>
+      </c>
+      <c r="D16" s="1" t="inlineStr">
+        <is>
+          <t>El sistema deberá mostrar un mensaje cuando la devolución haya sido registrada.</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>HU-002 – HU-002 - Registrar préstamo de libro</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Pendiente de definición y validación</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>RF-016</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Continuar proceso con datos correctos</t>
+        </is>
+      </c>
+      <c r="D17" s="1" t="inlineStr">
+        <is>
+          <t>El sistema deberá permitir continuar con el proceso cuando los datos sean correctos.</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>HU-002 – HU-002 - Registrar préstamo de libro</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Pendiente de definición y validación</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>RF-017</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Registrar mascota</t>
+        </is>
+      </c>
+      <c r="D18" s="1" t="inlineStr">
+        <is>
+          <t>El sistema deberá registrar mascota.</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>HU-002 – HU-002 - Registrar préstamo de libro</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Pendiente de validación</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>RF-018</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>El libro debe existir en el sistema</t>
+        </is>
+      </c>
+      <c r="D19" s="1" t="inlineStr">
+        <is>
+          <t>El sistema deberá el libro debe existir en el sistema.</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>HU-002 – HU-002 - Registrar préstamo de libro</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Pendiente de validación</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>RF-019</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>La devolución debe corresponder a un préstamo registrado</t>
+        </is>
+      </c>
+      <c r="D20" s="1" t="inlineStr">
+        <is>
+          <t>El sistema deberá la devolución debe corresponder a un préstamo registrado.</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>HU-002 – HU-002 - Registrar préstamo de libro</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Pendiente de validación</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>RF-020</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Todavía no se ha definido qué información específica debe actualizarse al registrar la devolución, cómo se manejarán las devoluciones realizadas fuera de plazo ni qué información deberá conservarse como evidencia de la operación</t>
+        </is>
+      </c>
+      <c r="D21" s="1" t="inlineStr">
+        <is>
+          <t>El sistema deberá todavía no se ha definido qué información específica debe actualizarse al registrar la devolución, cómo se manejarán las devoluciones realizadas fuera de plazo ni qué información deberá conservarse como evidencia de la operación.</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>HU-002 – HU-002 - Registrar préstamo de libro</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Pendiente de validación</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F12"/>
+  <autoFilter ref="A1:F21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>